<commit_message>
api updated and data file added
</commit_message>
<xml_diff>
--- a/public/Hotel Inventory Table Formatting.xlsx
+++ b/public/Hotel Inventory Table Formatting.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Rushi\internship manual\project\next_adwait_tour\public\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4AC3C91C-F06C-4D09-BC06-BB955BA9CEA8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5816319F-9836-4902-B46E-EEF60AA49E5B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="39" uniqueCount="29">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="46" uniqueCount="30">
   <si>
     <t>Hotel Name</t>
   </si>
@@ -107,6 +107,9 @@
   </si>
   <si>
     <t>OCP</t>
+  </si>
+  <si>
+    <t>exp-demo</t>
   </si>
 </sst>
 </file>
@@ -380,7 +383,7 @@
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:M15"/>
+  <dimension ref="A1:P15"/>
   <sheetFormatPr defaultColWidth="12.5703125" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="0.28515625" customWidth="1"/>
@@ -395,7 +398,7 @@
     <col min="13" max="13" width="11.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A1" s="1"/>
       <c r="B1" s="1" t="s">
         <v>18</v>
@@ -433,8 +436,17 @@
       <c r="M1" s="1" t="s">
         <v>25</v>
       </c>
-    </row>
-    <row r="2" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="N1" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="O1" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="P1" s="1" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="2" spans="1:16" x14ac:dyDescent="0.2">
       <c r="H2" s="1" t="s">
         <v>26</v>
       </c>
@@ -453,8 +465,17 @@
       <c r="M2" s="4">
         <v>46387</v>
       </c>
-    </row>
-    <row r="3" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="N2" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="O2" s="4">
+        <v>46211</v>
+      </c>
+      <c r="P2" s="4">
+        <v>46387</v>
+      </c>
+    </row>
+    <row r="3" spans="1:16" x14ac:dyDescent="0.2">
       <c r="H3" s="1" t="s">
         <v>3</v>
       </c>
@@ -473,8 +494,17 @@
       <c r="M3" s="1" t="s">
         <v>5</v>
       </c>
-    </row>
-    <row r="4" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="N3" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="O3" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="P3" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="4" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A4" s="1"/>
       <c r="B4" s="1" t="s">
         <v>6</v>
@@ -512,8 +542,17 @@
       <c r="M4" s="1">
         <v>17000</v>
       </c>
-    </row>
-    <row r="5" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="N4" s="1">
+        <v>13000</v>
+      </c>
+      <c r="O4" s="1">
+        <v>15000</v>
+      </c>
+      <c r="P4" s="1">
+        <v>17000</v>
+      </c>
+    </row>
+    <row r="5" spans="1:16" x14ac:dyDescent="0.2">
       <c r="G5" s="1" t="s">
         <v>9</v>
       </c>
@@ -535,13 +574,22 @@
       <c r="M5" s="1">
         <v>23500</v>
       </c>
-    </row>
-    <row r="6" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="N5" s="1">
+        <v>19500</v>
+      </c>
+      <c r="O5" s="1">
+        <v>21500</v>
+      </c>
+      <c r="P5" s="1">
+        <v>23500</v>
+      </c>
+    </row>
+    <row r="6" spans="1:16" x14ac:dyDescent="0.2">
       <c r="G6" s="1" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="7" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:16" x14ac:dyDescent="0.2">
       <c r="G7" s="1" t="s">
         <v>11</v>
       </c>
@@ -563,8 +611,17 @@
       <c r="M7" s="1">
         <v>6000</v>
       </c>
-    </row>
-    <row r="8" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="N7" s="1">
+        <v>3500</v>
+      </c>
+      <c r="O7" s="1">
+        <v>5000</v>
+      </c>
+      <c r="P7" s="1">
+        <v>6000</v>
+      </c>
+    </row>
+    <row r="8" spans="1:16" x14ac:dyDescent="0.2">
       <c r="G8" s="1" t="s">
         <v>12</v>
       </c>
@@ -586,8 +643,17 @@
       <c r="M8" s="1">
         <v>5000</v>
       </c>
-    </row>
-    <row r="9" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="N8" s="1">
+        <v>2500</v>
+      </c>
+      <c r="O8" s="1">
+        <v>4000</v>
+      </c>
+      <c r="P8" s="1">
+        <v>5000</v>
+      </c>
+    </row>
+    <row r="9" spans="1:16" x14ac:dyDescent="0.2">
       <c r="G9" s="1" t="s">
         <v>13</v>
       </c>
@@ -601,16 +667,25 @@
         <v>3500</v>
       </c>
       <c r="K9" s="1">
-        <v>1200</v>
+        <v>3700</v>
       </c>
       <c r="L9" s="1">
-        <v>2700</v>
+        <v>3700</v>
       </c>
       <c r="M9" s="1">
         <v>3700</v>
       </c>
-    </row>
-    <row r="10" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="N9" s="1">
+        <v>3700</v>
+      </c>
+      <c r="O9" s="1">
+        <v>3700</v>
+      </c>
+      <c r="P9" s="1">
+        <v>3700</v>
+      </c>
+    </row>
+    <row r="10" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A10" s="1"/>
       <c r="B10" s="1" t="s">
         <v>14</v>
@@ -649,7 +724,7 @@
         <v>13000</v>
       </c>
     </row>
-    <row r="11" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:16" x14ac:dyDescent="0.2">
       <c r="G11" s="1" t="s">
         <v>17</v>
       </c>
@@ -672,12 +747,12 @@
         <v>20000</v>
       </c>
     </row>
-    <row r="12" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:16" x14ac:dyDescent="0.2">
       <c r="G12" s="1" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="13" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:16" x14ac:dyDescent="0.2">
       <c r="G13" s="1" t="s">
         <v>11</v>
       </c>
@@ -700,7 +775,7 @@
         <v>4800</v>
       </c>
     </row>
-    <row r="14" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:16" x14ac:dyDescent="0.2">
       <c r="G14" s="1" t="s">
         <v>12</v>
       </c>
@@ -723,7 +798,7 @@
         <v>3800</v>
       </c>
     </row>
-    <row r="15" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:16" x14ac:dyDescent="0.2">
       <c r="G15" s="1" t="s">
         <v>13</v>
       </c>

</xml_diff>